<commit_message>
IPO Desk: Bombay Coated and Special Steels rebuilt from the RHP
RHP dated 21-Oct-2026 (FY26 and Q1 FY27 figures, offer, peers, dates).
Call stays Subscribe at the Rs 82 upper band; fair value Rs 103 / 110 /
126; reported P/E 16.9x, adjusted 17.4x. No longer provisional.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Sh3XfYSpHMqTXgPXQV3Xds
</commit_message>
<xml_diff>
--- a/ipo-analysis/companies/bombay-coated-and-special-steels-ltd/BOMBAY_COATED_AND_SPECIA_01_Screening.xlsx
+++ b/ipo-analysis/companies/bombay-coated-and-special-steels-ltd/BOMBAY_COATED_AND_SPECIA_01_Screening.xlsx
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>46050</v>
+        <v>46316</v>
       </c>
       <c r="D8" s="8" t="inlineStr"/>
     </row>
@@ -1032,7 +1032,7 @@
         </is>
       </c>
       <c r="C9" s="10" t="n">
-        <v>45930</v>
+        <v>46203</v>
       </c>
       <c r="D9" s="8" t="inlineStr"/>
     </row>
@@ -1111,7 +1111,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Price band, lot, issue size and dates from the NSE issue page (26-Oct-2026); financials from the DRHP dated 28-Jan-2026 because the RHP was not retrievable</t>
+          <t>none (all figures from the RHP; band, lot and size also on the NSE issue page)</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr"/>
@@ -1307,20 +1307,20 @@
         </is>
       </c>
       <c r="C5" s="16" t="n">
-        <v>590.875</v>
+        <v>755.259</v>
       </c>
       <c r="D5" s="16" t="n">
-        <v>755.259</v>
+        <v>1055.707</v>
       </c>
       <c r="E5" s="16" t="n">
-        <v>1055.707</v>
+        <v>1266.818</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>491.51</v>
+        <v>397.08</v>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>p. 279</t>
+          <t>p. 85</t>
         </is>
       </c>
     </row>
@@ -1331,20 +1331,20 @@
         </is>
       </c>
       <c r="C6" s="16" t="n">
-        <v>1.015</v>
+        <v>10.153</v>
       </c>
       <c r="D6" s="16" t="n">
-        <v>10.153</v>
+        <v>2.938</v>
       </c>
       <c r="E6" s="16" t="n">
-        <v>2.938</v>
+        <v>3.007</v>
       </c>
       <c r="F6" s="16" t="n">
-        <v>1.403</v>
+        <v>0.466</v>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>pp. 279, 329</t>
+          <t>pp. 85, 375</t>
         </is>
       </c>
     </row>
@@ -1355,20 +1355,20 @@
         </is>
       </c>
       <c r="C7" s="16" t="n">
-        <v>20.991</v>
+        <v>28.206</v>
       </c>
       <c r="D7" s="16" t="n">
-        <v>28.206</v>
+        <v>37.165</v>
       </c>
       <c r="E7" s="16" t="n">
-        <v>37.165</v>
+        <v>40.788</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>15.417</v>
+        <v>20.646</v>
       </c>
       <c r="G7" s="7" t="inlineStr">
         <is>
-          <t>p. 279</t>
+          <t>p. 85</t>
         </is>
       </c>
     </row>
@@ -1379,20 +1379,20 @@
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>4.461</v>
+        <v>5.703</v>
       </c>
       <c r="D8" s="16" t="n">
-        <v>5.703</v>
+        <v>7.124</v>
       </c>
       <c r="E8" s="16" t="n">
-        <v>7.124</v>
+        <v>8.023999999999999</v>
       </c>
       <c r="F8" s="16" t="n">
-        <v>2.888</v>
+        <v>4.857</v>
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>p. 279 (incl. earlier years)</t>
+          <t>p. 85 (incl. earlier years)</t>
         </is>
       </c>
     </row>
@@ -1403,20 +1403,20 @@
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>0.864</v>
+        <v>1.365</v>
       </c>
       <c r="D9" s="16" t="n">
-        <v>1.365</v>
+        <v>1.369</v>
       </c>
       <c r="E9" s="16" t="n">
-        <v>1.369</v>
+        <v>2.225</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>1.515</v>
+        <v>0.714</v>
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>p. 279</t>
+          <t>p. 85</t>
         </is>
       </c>
     </row>
@@ -1427,20 +1427,20 @@
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>15.666</v>
+        <v>21.138</v>
       </c>
       <c r="D10" s="16" t="n">
-        <v>21.138</v>
+        <v>28.672</v>
       </c>
       <c r="E10" s="16" t="n">
-        <v>28.672</v>
+        <v>30.539</v>
       </c>
       <c r="F10" s="16" t="n">
-        <v>11.014</v>
+        <v>15.075</v>
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>p. 279</t>
+          <t>p. 85</t>
         </is>
       </c>
     </row>
@@ -1451,20 +1451,20 @@
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>1.34</v>
+        <v>11.487</v>
       </c>
       <c r="D11" s="16" t="n">
-        <v>11.487</v>
+        <v>32.09</v>
       </c>
       <c r="E11" s="16" t="n">
-        <v>32.09</v>
+        <v>10.217</v>
       </c>
       <c r="F11" s="16" t="n">
-        <v>62.514</v>
+        <v>72.30500000000001</v>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>p. 280</t>
+          <t>p. 86</t>
         </is>
       </c>
     </row>
@@ -1488,7 +1488,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>pp. 32-33 (no sales to related parties)</t>
+          <t>pp. 89-92 (no sales to related parties)</t>
         </is>
       </c>
     </row>
@@ -1499,20 +1499,20 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>2.792</v>
+        <v>1.698</v>
       </c>
       <c r="D13" s="16" t="n">
-        <v>1.822</v>
+        <v>2.987</v>
       </c>
       <c r="E13" s="16" t="n">
-        <v>2.987</v>
+        <v>3.6</v>
       </c>
       <c r="F13" s="16" t="n">
-        <v>3.317</v>
+        <v>0.763</v>
       </c>
       <c r="G13" s="7" t="inlineStr">
         <is>
-          <t>pp. 32-33 (interest on promoter-family loans and rent paid to promoters)</t>
+          <t>pp. 89-92 (interest on promoter-family loans and rent paid to promoters)</t>
         </is>
       </c>
     </row>
@@ -1523,20 +1523,20 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>33.244</v>
+        <v>54.359</v>
       </c>
       <c r="D14" s="16" t="n">
-        <v>54.359</v>
+        <v>83.047</v>
       </c>
       <c r="E14" s="16" t="n">
-        <v>83.047</v>
+        <v>121.581</v>
       </c>
       <c r="F14" s="16" t="n">
-        <v>94.071</v>
+        <v>136.615</v>
       </c>
       <c r="G14" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
     </row>
@@ -1547,20 +1547,20 @@
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>80.334</v>
+        <v>106.151</v>
       </c>
       <c r="D15" s="16" t="n">
-        <v>106.151</v>
+        <v>136.729</v>
       </c>
       <c r="E15" s="16" t="n">
-        <v>136.729</v>
+        <v>128.922</v>
       </c>
       <c r="F15" s="16" t="n">
-        <v>115.818</v>
+        <v>165.41</v>
       </c>
       <c r="G15" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
     </row>
@@ -1571,20 +1571,20 @@
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>86.996</v>
+        <v>84.31999999999999</v>
       </c>
       <c r="D16" s="16" t="n">
-        <v>84.31999999999999</v>
+        <v>115.727</v>
       </c>
       <c r="E16" s="16" t="n">
-        <v>115.727</v>
+        <v>189.327</v>
       </c>
       <c r="F16" s="16" t="n">
-        <v>101.162</v>
+        <v>125.46</v>
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
     </row>
@@ -1595,20 +1595,20 @@
         </is>
       </c>
       <c r="C17" s="16" t="n">
-        <v>65.727</v>
+        <v>56.065</v>
       </c>
       <c r="D17" s="16" t="n">
-        <v>56.065</v>
+        <v>72.965</v>
       </c>
       <c r="E17" s="16" t="n">
-        <v>72.965</v>
+        <v>86.04900000000001</v>
       </c>
       <c r="F17" s="16" t="n">
-        <v>60.45</v>
+        <v>85.96599999999999</v>
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
     </row>
@@ -1632,7 +1632,7 @@
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>p. 31 (no contingent liabilities; capital commitments Rs 3.34 cr)</t>
+          <t>p. 87 (no contingent liabilities; capital commitments Rs 9.83 cr at Jun-26)</t>
         </is>
       </c>
     </row>
@@ -1656,7 +1656,7 @@
       </c>
       <c r="G19" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>0.1553</v>
+        <v>0.204</v>
       </c>
     </row>
     <row r="24">
@@ -1696,7 +1696,7 @@
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>0.6744</v>
+        <v>0.7133</v>
       </c>
     </row>
     <row r="25">
@@ -1706,7 +1706,7 @@
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>0.9061</v>
+        <v>0.8665</v>
       </c>
     </row>
     <row r="26">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>pp. 29, 94</t>
+          <t>pp. 99-100, 128</t>
         </is>
       </c>
       <c r="G5" s="27" t="inlineStr">
         <is>
-          <t>3:1 bonus (08-Jul-2025) is reflected: EPS 4.47 / 5.34 / 7.24 FY23-25 are on the post-bonus count of 3.96 crore shares. A further 9,00,091 shares were placed at Rs 88 on 28-Oct-2025 (4.05 crore shares now).</t>
+          <t>3:1 bonus (08-Jul-2025) and the 9,00,091-share placement at Rs 88 (28-Oct-2025) are reflected: FY26 EPS Rs 7.64 is on 3,99,79,764 weighted shares; 4,05,00,091 shares now.</t>
         </is>
       </c>
     </row>
@@ -2440,12 +2440,12 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>p. 280</t>
+          <t>p. 86</t>
         </is>
       </c>
       <c r="G6" s="27" t="inlineStr">
         <is>
-          <t>Operating cash flow Rs 1.34 / 11.49 / 32.09 cr FY23-25 against PAT Rs 15.67 / 21.14 / 28.67 cr: cumulative CFO/PAT 68.6% while revenue grew 34% a year. H1 FY26 CFO Rs 62.51 cr (PAT Rs 11.01 cr) as inventory and receivables were released; including H1, CFO exceeds PAT.</t>
+          <t>Operating cash flow Rs 11.49 / 32.09 / 10.22 cr FY24-26 against PAT Rs 21.14 / 28.67 / 30.54 cr: cumulative CFO/PAT 67.0% while revenue grew 30% a year and inventory rose Rs 73.6 cr in FY26. Q1 FY27 CFO Rs 72.31 cr (PAT Rs 15.08 cr) as inventory was released.</t>
         </is>
       </c>
     </row>
@@ -2477,12 +2477,12 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>p. 279</t>
+          <t>p. 85</t>
         </is>
       </c>
       <c r="G7" s="27" t="inlineStr">
         <is>
-          <t>Current tax 20.0% of cumulative FY23-25 PBT plus deferred tax (accelerated depreciation on new plants) 4.1%; income tax paid Rs 18.88 cr over three years.</t>
+          <t>Current tax 19.6% of cumulative FY24-26 PBT plus deferred tax (accelerated depreciation on new lines); income tax paid Rs 21.14 cr over three years.</t>
         </is>
       </c>
     </row>
@@ -2514,12 +2514,12 @@
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>pp. 32-33</t>
+          <t>pp. 89-92</t>
         </is>
       </c>
       <c r="G8" s="27" t="inlineStr">
         <is>
-          <t>Promoters and relatives lend the company Rs 25.75 cr (Sep-2025) at interest (Rs 2.52 cr of interest in FY25) and rent it two properties; managerial pay is modest (Rs 0.66 cr to three promoter directors in FY25). Related-party transactions 3.14% of FY25 revenue. Disclosed and typical of a promoter-funded company.</t>
+          <t>Promoters and relatives lend the company Rs 20.55 cr (Jun-26) at interest (Rs 3.08 cr in FY26) and rent it premises (Rs 0.52 cr in FY26); managerial pay Rs 0.66 cr to three promoter directors in FY26. Disclosed and typical of a promoter-funded company.</t>
         </is>
       </c>
     </row>
@@ -2551,12 +2551,12 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>pp. 27, 108</t>
+          <t>p. 117</t>
         </is>
       </c>
       <c r="G9" s="27" t="inlineStr">
         <is>
-          <t>Amount-based fresh issue (Rs 191 cr): Rs 125 cr repays borrowings, Rs 18 cr buys out Siemens equipment leases, balance GCP (cap 25%). No fixed share count, so no objects floor.</t>
+          <t>Amount-based fresh issue (Rs 183.06 cr): Rs 125 cr repays borrowings, Rs 15.77 cr buys out Siemens equipment leases, balance GCP (cap 25%). No fixed share count, so no objects floor.</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>p. 278</t>
+          <t>p. 84</t>
         </is>
       </c>
       <c r="G11" s="27" t="inlineStr">
@@ -2654,12 +2654,12 @@
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>pp. 30-31, 37</t>
+          <t>pp. 34-35</t>
         </is>
       </c>
       <c r="G12" s="27" t="inlineStr">
         <is>
-          <t>JSW Steel Coated Products supplied 90.61% of FY25 steel coils (authorised service partner since 2021); appliances 81.80% of FY25 product revenue; top customer (Amber Enterprises) 15.53% and top-10 67.44%. Typical of a service centre tied to one mill and the appliance PLI ecosystem.</t>
+          <t>JSW Steel Coated Products supplied 86.65% of FY26 steel coils (85.13% in Q1 FY27); appliances 86.54% of FY26 product revenue; top customer (Amber Enterprises) 20.40% and top-10 71.33% of FY26 revenue. Typical of a service centre tied to one mill and the appliance PLI ecosystem.</t>
         </is>
       </c>
     </row>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>p. 31</t>
+          <t>p. 87</t>
         </is>
       </c>
       <c r="G13" s="27" t="inlineStr">
         <is>
-          <t>No contingent liabilities; capital commitments Rs 3.34 cr (Sep-2025).</t>
+          <t>No contingent liabilities; capital commitments Rs 9.83 cr (Jun-26).</t>
         </is>
       </c>
     </row>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>pp. 29, 88</t>
+          <t>p. 82</t>
         </is>
       </c>
       <c r="G15" s="27" t="inlineStr">
         <is>
-          <t>Shah Shah &amp; Shah (peer-reviewed); no qualifications. A previous auditor resigned in Aug-2021, before the current growth phase.</t>
+          <t>Shah Shah &amp; Shah (peer-reviewed); no qualifications.</t>
         </is>
       </c>
     </row>
@@ -2798,12 +2798,12 @@
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>pp. 44-46</t>
+          <t>p. 32</t>
         </is>
       </c>
       <c r="G16" s="27" t="inlineStr">
         <is>
-          <t>25 delayed RoC filings over five years and a 2021 allotment to a promoter (for the Bombay Steels business transfer) filed with the wrong form and without MGT-14; compounding / adjudication application pending before the RoC. Procedural, rectified with additional fees; no penalty yet.</t>
+          <t>25 delayed RoC filings over five years and a 2021 allotment to a promoter filed with the wrong form; adjudication application (06-Jan-2026) still pending before the RoC. Procedural; no penalty yet.</t>
         </is>
       </c>
     </row>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>p. 108</t>
+          <t>p. 117</t>
         </is>
       </c>
       <c r="G17" s="27" t="inlineStr">
         <is>
-          <t>Fresh issue Rs 191 cr: monitoring agency mandatory; to be named in the RHP.</t>
+          <t>Monitoring agency appointed for the use of proceeds.</t>
         </is>
       </c>
     </row>
@@ -2936,14 +2936,10 @@
           <t>OPEN</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr">
-        <is>
-          <t>p. 434</t>
-        </is>
-      </c>
+      <c r="F20" s="7" t="inlineStr"/>
       <c r="G20" s="27" t="inlineStr">
         <is>
-          <t>Smart Horizon Capital Advisors: past-issue track record is referenced to its website and not compiled in this run.</t>
+          <t>Smart Horizon Capital Advisors: track record of past issues not compiled in this run.</t>
         </is>
       </c>
     </row>

</xml_diff>